<commit_message>
Ship Ver 1.4.2: read catalogs from a local mirror, and wait for background work before the window closes.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/data_tables/三路电阻.xlsx
+++ b/templates/data_tables/三路电阻.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ikaruga/Desktop/Reach/report creator/templates/data_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/材料实验室b/车载电子/report_creator/data_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD59A55-C58A-2944-8136-6C53198E015D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9E9C2F-FEC3-AD4F-BE95-9F4DC14318DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <r>
       <t>绝缘电阻
@@ -101,6 +101,14 @@
   </si>
   <si>
     <t>试验后after test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>上限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>下限</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -463,21 +471,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="19.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="23.796875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4">
+    <row r="1" spans="1:4">
       <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="2:4" ht="30">
+    <row r="2" spans="1:4" ht="30">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -488,6 +496,16 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:D1"/>

</xml_diff>